<commit_message>
Modified the number of extracted parameters
</commit_message>
<xml_diff>
--- a/04_Data Extraction/Data_Extraction_Form.xlsx
+++ b/04_Data Extraction/Data_Extraction_Form.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:AP3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -602,27 +602,27 @@
           <t>Partitioning Memory</t>
         </is>
       </c>
-      <c r="W1" s="5" t="inlineStr">
+      <c r="V1" s="5" t="inlineStr">
         <is>
           <t>Handling Traps and Interrupts</t>
         </is>
       </c>
-      <c r="AA1" s="6" t="inlineStr">
+      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>I/O Virtualization</t>
         </is>
       </c>
-      <c r="AC1" s="7" t="inlineStr">
+      <c r="AA1" s="7" t="inlineStr">
         <is>
           <t>Start-Up Sequence and Partition Switch</t>
         </is>
       </c>
-      <c r="AG1" s="8" t="inlineStr">
+      <c r="AE1" s="8" t="inlineStr">
         <is>
           <t>Services to Partitions</t>
         </is>
       </c>
-      <c r="AK1" s="9" t="inlineStr">
+      <c r="AI1" s="9" t="inlineStr">
         <is>
           <t>Impact on Performance</t>
         </is>
@@ -726,125 +726,115 @@
       </c>
       <c r="T2" s="10" t="inlineStr">
         <is>
-          <t>HW-based isolation (Configuration strategy)</t>
+          <t>HW-based isolation</t>
         </is>
       </c>
       <c r="U2" s="10" t="inlineStr">
         <is>
-          <t>HW-based isolation (Protection mechanism)</t>
+          <t>SW-based isolation</t>
         </is>
       </c>
       <c r="V2" s="10" t="inlineStr">
         <is>
-          <t>SW-based isolation</t>
+          <t>Interrupt handling</t>
         </is>
       </c>
       <c r="W2" s="10" t="inlineStr">
         <is>
-          <t>Interrupt handling (Strategy)</t>
+          <t>Privilege emulation</t>
         </is>
       </c>
       <c r="X2" s="10" t="inlineStr">
         <is>
-          <t>Interrupt handling (Mechanism)</t>
+          <t>Exception handling</t>
         </is>
       </c>
       <c r="Y2" s="10" t="inlineStr">
         <is>
-          <t>Privilege emulation</t>
+          <t>Peripheral virtualization strategy</t>
         </is>
       </c>
       <c r="Z2" s="10" t="inlineStr">
         <is>
-          <t>Exception handling</t>
+          <t>Support for shared peripherals</t>
         </is>
       </c>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>Peripheral virtualization strategy</t>
+          <t>Boot order</t>
         </is>
       </c>
       <c r="AB2" s="10" t="inlineStr">
         <is>
-          <t>Support for shared peripherals</t>
+          <t>Partition creation</t>
         </is>
       </c>
       <c r="AC2" s="10" t="inlineStr">
         <is>
-          <t>Boot order</t>
+          <t>Partition switch</t>
         </is>
       </c>
       <c r="AD2" s="10" t="inlineStr">
         <is>
-          <t>Partition creation</t>
+          <t>Partition scheduling</t>
         </is>
       </c>
       <c r="AE2" s="10" t="inlineStr">
         <is>
-          <t>Partition switch</t>
+          <t>Task handling inside partitions</t>
         </is>
       </c>
       <c r="AF2" s="10" t="inlineStr">
         <is>
-          <t>Partition scheduling</t>
+          <t>Shared memory regions across partitions</t>
         </is>
       </c>
       <c r="AG2" s="10" t="inlineStr">
         <is>
-          <t>Task handling inside partitions</t>
+          <t>Inter-partition communication</t>
         </is>
       </c>
       <c r="AH2" s="10" t="inlineStr">
         <is>
-          <t>Shared memory regions across partitions</t>
+          <t>Service interface</t>
         </is>
       </c>
       <c r="AI2" s="10" t="inlineStr">
         <is>
-          <t>Inter-partition communication</t>
+          <t>Total execution time overhead</t>
         </is>
       </c>
       <c r="AJ2" s="10" t="inlineStr">
         <is>
-          <t>Service interface</t>
+          <t>Context switch overhead</t>
         </is>
       </c>
       <c r="AK2" s="10" t="inlineStr">
         <is>
-          <t>Total execution time overhead</t>
+          <t>Hypercall latency</t>
         </is>
       </c>
       <c r="AL2" s="10" t="inlineStr">
         <is>
-          <t>Context switch overhead</t>
+          <t>Interrupt handling latency</t>
         </is>
       </c>
       <c r="AM2" s="10" t="inlineStr">
         <is>
-          <t>Hypercall latency</t>
+          <t>I/O access latency</t>
         </is>
       </c>
       <c r="AN2" s="10" t="inlineStr">
         <is>
-          <t>Interrupt handling latency</t>
+          <t>HW resource overhead</t>
         </is>
       </c>
       <c r="AO2" s="10" t="inlineStr">
         <is>
-          <t>I/O access latency</t>
+          <t>Power overhead</t>
         </is>
       </c>
       <c r="AP2" s="10" t="inlineStr">
-        <is>
-          <t>HW resource overhead</t>
-        </is>
-      </c>
-      <c r="AQ2" s="10" t="inlineStr">
-        <is>
-          <t>Power overhead</t>
-        </is>
-      </c>
-      <c r="AR2" s="10" t="inlineStr">
         <is>
           <t>Memory footprint</t>
         </is>
@@ -983,12 +973,12 @@
       </c>
       <c r="AA3" s="11" t="inlineStr">
         <is>
-          <t>RQ3</t>
+          <t>RQ4</t>
         </is>
       </c>
       <c r="AB3" s="11" t="inlineStr">
         <is>
-          <t>RQ3</t>
+          <t>RQ4</t>
         </is>
       </c>
       <c r="AC3" s="11" t="inlineStr">
@@ -1023,12 +1013,12 @@
       </c>
       <c r="AI3" s="11" t="inlineStr">
         <is>
-          <t>RQ4</t>
+          <t>RQ5</t>
         </is>
       </c>
       <c r="AJ3" s="11" t="inlineStr">
         <is>
-          <t>RQ4</t>
+          <t>RQ5</t>
         </is>
       </c>
       <c r="AK3" s="11" t="inlineStr">
@@ -1057,16 +1047,6 @@
         </is>
       </c>
       <c r="AP3" s="11" t="inlineStr">
-        <is>
-          <t>RQ5</t>
-        </is>
-      </c>
-      <c r="AQ3" s="11" t="inlineStr">
-        <is>
-          <t>RQ5</t>
-        </is>
-      </c>
-      <c r="AR3" s="11" t="inlineStr">
         <is>
           <t>RQ5</t>
         </is>
@@ -1075,14 +1055,14 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="T1:V1"/>
     <mergeCell ref="M1:S1"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="AA1:AB1"/>
-    <mergeCell ref="AK1:AR1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="AE1:AH1"/>
+    <mergeCell ref="Y1:Z1"/>
+    <mergeCell ref="AI1:AP1"/>
+    <mergeCell ref="AA1:AD1"/>
+    <mergeCell ref="V1:X1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1094,7 +1074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR21"/>
+  <dimension ref="A1:AP21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1164,27 +1144,27 @@
           <t>Partitioning Memory</t>
         </is>
       </c>
-      <c r="W1" s="5" t="inlineStr">
+      <c r="V1" s="5" t="inlineStr">
         <is>
           <t>Handling Traps and Interrupts</t>
         </is>
       </c>
-      <c r="AA1" s="6" t="inlineStr">
+      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>I/O Virtualization</t>
         </is>
       </c>
-      <c r="AC1" s="7" t="inlineStr">
+      <c r="AA1" s="7" t="inlineStr">
         <is>
           <t>Start-Up Sequence and Partition Switch</t>
         </is>
       </c>
-      <c r="AG1" s="8" t="inlineStr">
+      <c r="AE1" s="8" t="inlineStr">
         <is>
           <t>Services to Partitions</t>
         </is>
       </c>
-      <c r="AK1" s="9" t="inlineStr">
+      <c r="AI1" s="9" t="inlineStr">
         <is>
           <t>Impact on Performance</t>
         </is>
@@ -1288,125 +1268,115 @@
       </c>
       <c r="T2" s="10" t="inlineStr">
         <is>
-          <t>HW-based isolation (Configuration strategy)</t>
+          <t>HW-based isolation</t>
         </is>
       </c>
       <c r="U2" s="10" t="inlineStr">
         <is>
-          <t>HW-based isolation (Protection mechanism)</t>
+          <t>SW-based isolation</t>
         </is>
       </c>
       <c r="V2" s="10" t="inlineStr">
         <is>
-          <t>SW-based isolation</t>
+          <t>Interrupt handling</t>
         </is>
       </c>
       <c r="W2" s="10" t="inlineStr">
         <is>
-          <t>Interrupt handling (Strategy)</t>
+          <t>Privilege emulation</t>
         </is>
       </c>
       <c r="X2" s="10" t="inlineStr">
         <is>
-          <t>Interrupt handling (Mechanism)</t>
+          <t>Exception handling</t>
         </is>
       </c>
       <c r="Y2" s="10" t="inlineStr">
         <is>
-          <t>Privilege emulation</t>
+          <t>Peripheral virtualization strategy</t>
         </is>
       </c>
       <c r="Z2" s="10" t="inlineStr">
         <is>
-          <t>Exception handling</t>
+          <t>Support for shared peripherals</t>
         </is>
       </c>
       <c r="AA2" s="10" t="inlineStr">
         <is>
-          <t>Peripheral virtualization strategy</t>
+          <t>Boot order</t>
         </is>
       </c>
       <c r="AB2" s="10" t="inlineStr">
         <is>
-          <t>Support for shared peripherals</t>
+          <t>Partition creation</t>
         </is>
       </c>
       <c r="AC2" s="10" t="inlineStr">
         <is>
-          <t>Boot order</t>
+          <t>Partition switch</t>
         </is>
       </c>
       <c r="AD2" s="10" t="inlineStr">
         <is>
-          <t>Partition creation</t>
+          <t>Partition scheduling</t>
         </is>
       </c>
       <c r="AE2" s="10" t="inlineStr">
         <is>
-          <t>Partition switch</t>
+          <t>Task handling inside partitions</t>
         </is>
       </c>
       <c r="AF2" s="10" t="inlineStr">
         <is>
-          <t>Partition scheduling</t>
+          <t>Shared memory regions across partitions</t>
         </is>
       </c>
       <c r="AG2" s="10" t="inlineStr">
         <is>
-          <t>Task handling inside partitions</t>
+          <t>Inter-partition communication</t>
         </is>
       </c>
       <c r="AH2" s="10" t="inlineStr">
         <is>
-          <t>Shared memory regions across partitions</t>
+          <t>Service interface</t>
         </is>
       </c>
       <c r="AI2" s="10" t="inlineStr">
         <is>
-          <t>Inter-partition communication</t>
+          <t>Total execution time overhead</t>
         </is>
       </c>
       <c r="AJ2" s="10" t="inlineStr">
         <is>
-          <t>Service interface</t>
+          <t>Context switch overhead</t>
         </is>
       </c>
       <c r="AK2" s="10" t="inlineStr">
         <is>
-          <t>Total execution time overhead</t>
+          <t>Hypercall latency</t>
         </is>
       </c>
       <c r="AL2" s="10" t="inlineStr">
         <is>
-          <t>Context switch overhead</t>
+          <t>Interrupt handling latency</t>
         </is>
       </c>
       <c r="AM2" s="10" t="inlineStr">
         <is>
-          <t>Hypercall latency</t>
+          <t>I/O access latency</t>
         </is>
       </c>
       <c r="AN2" s="10" t="inlineStr">
         <is>
-          <t>Interrupt handling latency</t>
+          <t>HW resource overhead</t>
         </is>
       </c>
       <c r="AO2" s="10" t="inlineStr">
         <is>
-          <t>I/O access latency</t>
+          <t>Power overhead</t>
         </is>
       </c>
       <c r="AP2" s="10" t="inlineStr">
-        <is>
-          <t>HW resource overhead</t>
-        </is>
-      </c>
-      <c r="AQ2" s="10" t="inlineStr">
-        <is>
-          <t>Power overhead</t>
-        </is>
-      </c>
-      <c r="AR2" s="10" t="inlineStr">
         <is>
           <t>Memory footprint</t>
         </is>
@@ -1508,87 +1478,87 @@
       </c>
       <c r="T3" s="12" t="inlineStr">
         <is>
+          <t>MPU (static)</t>
+        </is>
+      </c>
+      <c r="U3" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V3" s="12" t="inlineStr">
+        <is>
+          <t>Virtualization: Dedicated core for interrupt handling and interrupt injection</t>
+        </is>
+      </c>
+      <c r="W3" s="12" t="inlineStr">
+        <is>
+          <t>Hypercall</t>
+        </is>
+      </c>
+      <c r="X3" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="Y3" s="12" t="inlineStr">
+        <is>
+          <t>Driver partition</t>
+        </is>
+      </c>
+      <c r="Z3" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA3" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="AB3" s="12" t="inlineStr">
+        <is>
           <t>Static</t>
         </is>
       </c>
-      <c r="U3" s="12" t="inlineStr">
-        <is>
-          <t>MPU</t>
-        </is>
-      </c>
-      <c r="V3" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W3" s="12" t="inlineStr">
-        <is>
-          <t>Virtualization</t>
-        </is>
-      </c>
-      <c r="X3" s="12" t="inlineStr">
-        <is>
-          <t>Dedicated core for interrupt handling and interrupt injection</t>
-        </is>
-      </c>
-      <c r="Y3" s="12" t="inlineStr">
-        <is>
-          <t>Hypercall</t>
-        </is>
-      </c>
-      <c r="Z3" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AA3" s="12" t="inlineStr">
-        <is>
-          <t>Driver partition</t>
-        </is>
-      </c>
-      <c r="AB3" s="12" t="inlineStr">
+      <c r="AC3" s="12" t="inlineStr">
+        <is>
+          <t>N/A (1 VM/core)</t>
+        </is>
+      </c>
+      <c r="AD3" s="12" t="inlineStr">
+        <is>
+          <t>N/A (1 VM/core)</t>
+        </is>
+      </c>
+      <c r="AE3" s="12" t="inlineStr">
+        <is>
+          <t>Not discussed</t>
+        </is>
+      </c>
+      <c r="AF3" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AC3" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD3" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE3" s="12" t="inlineStr">
-        <is>
-          <t>N/A (1 VM/core)</t>
-        </is>
-      </c>
-      <c r="AF3" s="12" t="inlineStr">
-        <is>
-          <t>N/A (1 VM/core)</t>
-        </is>
-      </c>
       <c r="AG3" s="12" t="inlineStr">
         <is>
-          <t>Not discussed</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AH3" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Resource-scoped interfaces</t>
         </is>
       </c>
       <c r="AI3" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ3" s="12" t="inlineStr">
         <is>
-          <t>Resource-scoped interfaces</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK3" s="12" t="inlineStr">
@@ -1603,30 +1573,20 @@
       </c>
       <c r="AM3" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AN3" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO3" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AP3" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ3" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR3" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1728,107 +1688,107 @@
       </c>
       <c r="T4" s="12" t="inlineStr">
         <is>
-          <t>Dynamic</t>
+          <t>MPU (dynamic)</t>
         </is>
       </c>
       <c r="U4" s="12" t="inlineStr">
         <is>
-          <t>MPU</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V4" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Partitioning: Virtualization layer-mediated interrupt forwarding</t>
         </is>
       </c>
       <c r="W4" s="12" t="inlineStr">
         <is>
-          <t>Partitioning</t>
+          <t>Hypercall</t>
         </is>
       </c>
       <c r="X4" s="12" t="inlineStr">
         <is>
-          <t>Virtualization layer-mediated interrupt forwarding</t>
+          <t>ARINC/AUTOSAR specifications</t>
         </is>
       </c>
       <c r="Y4" s="12" t="inlineStr">
         <is>
-          <t>Hypercall</t>
+          <t>DDA + Driver partition</t>
         </is>
       </c>
       <c r="Z4" s="12" t="inlineStr">
         <is>
-          <t>ARINC/AUTOSAR specifications</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AA4" s="12" t="inlineStr">
         <is>
-          <t>DDA + Driver partition</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="AB4" s="12" t="inlineStr">
         <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="AC4" s="12" t="inlineStr">
+        <is>
+          <t>Static time partitioning</t>
+        </is>
+      </c>
+      <c r="AD4" s="12" t="inlineStr">
+        <is>
+          <t>Static time partitioning</t>
+        </is>
+      </c>
+      <c r="AE4" s="12" t="inlineStr">
+        <is>
+          <t>Managed by virtualization layer</t>
+        </is>
+      </c>
+      <c r="AF4" s="12" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AC4" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD4" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE4" s="12" t="inlineStr">
-        <is>
-          <t>Static time partitioning</t>
-        </is>
-      </c>
-      <c r="AF4" s="12" t="inlineStr">
-        <is>
-          <t>Static time partitioning</t>
-        </is>
-      </c>
       <c r="AG4" s="12" t="inlineStr">
         <is>
-          <t>Managed by virtualization layer</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AH4" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Standard middleware APIs</t>
         </is>
       </c>
       <c r="AI4" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ4" s="12" t="inlineStr">
         <is>
-          <t>Standard middleware APIs</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AK4" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AL4" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AM4" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AN4" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO4" s="12" t="inlineStr">
@@ -1837,16 +1797,6 @@
         </is>
       </c>
       <c r="AP4" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ4" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR4" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1948,87 +1898,87 @@
       </c>
       <c r="T5" s="12" t="inlineStr">
         <is>
+          <t>SMPU (static)</t>
+        </is>
+      </c>
+      <c r="U5" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V5" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="W5" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="X5" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="Y5" s="12" t="inlineStr">
+        <is>
+          <t>Driver partition</t>
+        </is>
+      </c>
+      <c r="Z5" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA5" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="AB5" s="12" t="inlineStr">
+        <is>
           <t>Static</t>
         </is>
       </c>
-      <c r="U5" s="12" t="inlineStr">
-        <is>
-          <t>SMPU</t>
-        </is>
-      </c>
-      <c r="V5" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W5" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="X5" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="Y5" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="Z5" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AA5" s="12" t="inlineStr">
-        <is>
-          <t>Driver partition</t>
-        </is>
-      </c>
-      <c r="AB5" s="12" t="inlineStr">
+      <c r="AC5" s="12" t="inlineStr">
+        <is>
+          <t>Static time partitioning</t>
+        </is>
+      </c>
+      <c r="AD5" s="12" t="inlineStr">
+        <is>
+          <t>Static time partitioning</t>
+        </is>
+      </c>
+      <c r="AE5" s="12" t="inlineStr">
+        <is>
+          <t>Not discussed</t>
+        </is>
+      </c>
+      <c r="AF5" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AC5" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD5" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE5" s="12" t="inlineStr">
-        <is>
-          <t>Static time partitioning</t>
-        </is>
-      </c>
-      <c r="AF5" s="12" t="inlineStr">
-        <is>
-          <t>Static time partitioning</t>
-        </is>
-      </c>
       <c r="AG5" s="12" t="inlineStr">
         <is>
-          <t>Not discussed</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AH5" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Standard middleware APIs</t>
         </is>
       </c>
       <c r="AI5" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ5" s="12" t="inlineStr">
         <is>
-          <t>Standard middleware APIs</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK5" s="12" t="inlineStr">
@@ -2043,30 +1993,20 @@
       </c>
       <c r="AM5" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AN5" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO5" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AP5" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ5" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR5" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2168,92 +2108,92 @@
       </c>
       <c r="T6" s="12" t="inlineStr">
         <is>
-          <t>Dynamic</t>
+          <t>MPU (dynamic)</t>
         </is>
       </c>
       <c r="U6" s="12" t="inlineStr">
         <is>
-          <t>MPU</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V6" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Virtualization: Virtual interrupt injection</t>
         </is>
       </c>
       <c r="W6" s="12" t="inlineStr">
         <is>
-          <t>Virtualization</t>
+          <t>Hypercall</t>
         </is>
       </c>
       <c r="X6" s="12" t="inlineStr">
         <is>
-          <t>Virtual interrupt injection</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="Y6" s="12" t="inlineStr">
         <is>
-          <t>Hypercall</t>
+          <t>DDA + Driver partition</t>
         </is>
       </c>
       <c r="Z6" s="12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA6" s="12" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="AA6" s="12" t="inlineStr">
-        <is>
-          <t>DDA + Driver partition</t>
-        </is>
-      </c>
       <c r="AB6" s="12" t="inlineStr">
         <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="AC6" s="12" t="inlineStr">
+        <is>
+          <t>Fixed-priority preemptive</t>
+        </is>
+      </c>
+      <c r="AD6" s="12" t="inlineStr">
+        <is>
+          <t>Fixed-priority preemptive</t>
+        </is>
+      </c>
+      <c r="AE6" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF6" s="12" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AC6" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD6" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE6" s="12" t="inlineStr">
-        <is>
-          <t>Fixed-priority preemptive</t>
-        </is>
-      </c>
-      <c r="AF6" s="12" t="inlineStr">
-        <is>
-          <t>Fixed-priority preemptive</t>
-        </is>
-      </c>
       <c r="AG6" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AH6" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Proprietary hypervisor APIs</t>
         </is>
       </c>
       <c r="AI6" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ6" s="12" t="inlineStr">
         <is>
-          <t>Proprietary hypervisor APIs</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK6" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AL6" s="12" t="inlineStr">
@@ -2263,12 +2203,12 @@
       </c>
       <c r="AM6" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AN6" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO6" s="12" t="inlineStr">
@@ -2277,16 +2217,6 @@
         </is>
       </c>
       <c r="AP6" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ6" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR6" s="12" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -2388,72 +2318,72 @@
       </c>
       <c r="T7" s="12" t="inlineStr">
         <is>
+          <t>MPU (static)</t>
+        </is>
+      </c>
+      <c r="U7" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V7" s="12" t="inlineStr">
+        <is>
+          <t>Partitioning: Virtualization layer-mediated interrupt forwarding</t>
+        </is>
+      </c>
+      <c r="W7" s="12" t="inlineStr">
+        <is>
+          <t>Trap-and-emulate</t>
+        </is>
+      </c>
+      <c r="X7" s="12" t="inlineStr">
+        <is>
+          <t>3-class routing</t>
+        </is>
+      </c>
+      <c r="Y7" s="12" t="inlineStr">
+        <is>
+          <t>DDA + Trap-and-emulate (full virtualization)</t>
+        </is>
+      </c>
+      <c r="Z7" s="12" t="inlineStr">
+        <is>
+          <t>Not evaluated</t>
+        </is>
+      </c>
+      <c r="AA7" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="AB7" s="12" t="inlineStr">
+        <is>
           <t>Static</t>
         </is>
       </c>
-      <c r="U7" s="12" t="inlineStr">
-        <is>
-          <t>MPU</t>
-        </is>
-      </c>
-      <c r="V7" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W7" s="12" t="inlineStr">
-        <is>
-          <t>Partitioning</t>
-        </is>
-      </c>
-      <c r="X7" s="12" t="inlineStr">
-        <is>
-          <t>Virtualization layer-mediated interrupt forwarding</t>
-        </is>
-      </c>
-      <c r="Y7" s="12" t="inlineStr">
-        <is>
-          <t>Trap-and-emulate</t>
-        </is>
-      </c>
-      <c r="Z7" s="12" t="inlineStr">
-        <is>
-          <t>3-class routing</t>
-        </is>
-      </c>
-      <c r="AA7" s="12" t="inlineStr">
-        <is>
-          <t>DDA + Trap-and-emulate (full virtualization)</t>
-        </is>
-      </c>
-      <c r="AB7" s="12" t="inlineStr">
-        <is>
-          <t>Not evaluated</t>
-        </is>
-      </c>
       <c r="AC7" s="12" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>N/A (1 VM/core)</t>
         </is>
       </c>
       <c r="AD7" s="12" t="inlineStr">
         <is>
-          <t>Static</t>
+          <t>N/A (1 VM/core)</t>
         </is>
       </c>
       <c r="AE7" s="12" t="inlineStr">
         <is>
-          <t>N/A (1 VM/core)</t>
+          <t>Not discussed</t>
         </is>
       </c>
       <c r="AF7" s="12" t="inlineStr">
         <is>
-          <t>N/A (1 VM/core)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AG7" s="12" t="inlineStr">
         <is>
-          <t>Not discussed</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH7" s="12" t="inlineStr">
@@ -2463,12 +2393,12 @@
       </c>
       <c r="AI7" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ7" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK7" s="12" t="inlineStr">
@@ -2478,35 +2408,25 @@
       </c>
       <c r="AL7" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AM7" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AN7" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO7" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AP7" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ7" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR7" s="12" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -2608,72 +2528,72 @@
       </c>
       <c r="T8" s="12" t="inlineStr">
         <is>
+          <t>TrustZone-M (static)</t>
+        </is>
+      </c>
+      <c r="U8" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V8" s="12" t="inlineStr">
+        <is>
+          <t>Direct Access: HW guest attribution</t>
+        </is>
+      </c>
+      <c r="W8" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="X8" s="12" t="inlineStr">
+        <is>
+          <t>HPV-centralized</t>
+        </is>
+      </c>
+      <c r="Y8" s="12" t="inlineStr">
+        <is>
+          <t>DDA (pass-through)</t>
+        </is>
+      </c>
+      <c r="Z8" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA8" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="AB8" s="12" t="inlineStr">
+        <is>
           <t>Static</t>
         </is>
       </c>
-      <c r="U8" s="12" t="inlineStr">
-        <is>
-          <t>TrustZone-M</t>
-        </is>
-      </c>
-      <c r="V8" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W8" s="12" t="inlineStr">
-        <is>
-          <t>Direct Access</t>
-        </is>
-      </c>
-      <c r="X8" s="12" t="inlineStr">
-        <is>
-          <t>HW guest attribution</t>
-        </is>
-      </c>
-      <c r="Y8" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z8" s="12" t="inlineStr">
-        <is>
-          <t>HPV-centralized</t>
-        </is>
-      </c>
-      <c r="AA8" s="12" t="inlineStr">
-        <is>
-          <t>DDA (pass-through)</t>
-        </is>
-      </c>
-      <c r="AB8" s="12" t="inlineStr">
+      <c r="AC8" s="12" t="inlineStr">
+        <is>
+          <t>Asymmetric scheduling - SC: N/A (1 VM/core) - MC</t>
+        </is>
+      </c>
+      <c r="AD8" s="12" t="inlineStr">
+        <is>
+          <t>Asymmetric scheduling</t>
+        </is>
+      </c>
+      <c r="AE8" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF8" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AC8" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD8" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE8" s="12" t="inlineStr">
-        <is>
-          <t>Asymmetric scheduling - SC: N/A (1 VM/core) - MC</t>
-        </is>
-      </c>
-      <c r="AF8" s="12" t="inlineStr">
-        <is>
-          <t>Asymmetric scheduling</t>
-        </is>
-      </c>
       <c r="AG8" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH8" s="12" t="inlineStr">
@@ -2683,24 +2603,24 @@
       </c>
       <c r="AI8" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AJ8" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK8" s="12" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AL8" s="12" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="AL8" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="AM8" s="12" t="inlineStr">
         <is>
           <t>—</t>
@@ -2708,7 +2628,7 @@
       </c>
       <c r="AN8" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO8" s="12" t="inlineStr">
@@ -2717,16 +2637,6 @@
         </is>
       </c>
       <c r="AP8" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ8" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR8" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2843,72 +2753,72 @@
       </c>
       <c r="W9" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>None</t>
         </is>
       </c>
       <c r="X9" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="Y9" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>HW I/O virtualization</t>
         </is>
       </c>
       <c r="Z9" s="12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA9" s="12" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="AA9" s="12" t="inlineStr">
-        <is>
-          <t>HW I/O virtualization</t>
-        </is>
-      </c>
       <c r="AB9" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Static</t>
         </is>
       </c>
       <c r="AC9" s="12" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>N/A (1 VM/core)</t>
         </is>
       </c>
       <c r="AD9" s="12" t="inlineStr">
         <is>
-          <t>Static</t>
+          <t>N/A (1 VM/core)</t>
         </is>
       </c>
       <c r="AE9" s="12" t="inlineStr">
         <is>
-          <t>N/A (1 VM/core)</t>
+          <t>Delegated to tenant</t>
         </is>
       </c>
       <c r="AF9" s="12" t="inlineStr">
         <is>
-          <t>N/A (1 VM/core)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AG9" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH9" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Resource-scoped interfaces</t>
         </is>
       </c>
       <c r="AI9" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ9" s="12" t="inlineStr">
         <is>
-          <t>Resource-scoped interfaces</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK9" s="12" t="inlineStr">
@@ -2923,12 +2833,12 @@
       </c>
       <c r="AM9" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AN9" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AO9" s="12" t="inlineStr">
@@ -2937,16 +2847,6 @@
         </is>
       </c>
       <c r="AP9" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="AQ9" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="AR9" s="12" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -3048,87 +2948,87 @@
       </c>
       <c r="T10" s="12" t="inlineStr">
         <is>
+          <t>HW VMM (static)</t>
+        </is>
+      </c>
+      <c r="U10" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V10" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W10" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="X10" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="Y10" s="12" t="inlineStr">
+        <is>
+          <t>HW I/O virtualization</t>
+        </is>
+      </c>
+      <c r="Z10" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA10" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="AB10" s="12" t="inlineStr">
+        <is>
           <t>Static</t>
         </is>
       </c>
-      <c r="U10" s="12" t="inlineStr">
-        <is>
-          <t>HW VMM</t>
-        </is>
-      </c>
-      <c r="V10" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W10" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X10" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Y10" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z10" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AA10" s="12" t="inlineStr">
-        <is>
-          <t>HW I/O virtualization</t>
-        </is>
-      </c>
-      <c r="AB10" s="12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="AC10" s="12" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>N/A (1 VM/core)</t>
         </is>
       </c>
       <c r="AD10" s="12" t="inlineStr">
         <is>
-          <t>Static</t>
+          <t>N/A (1 VM/core)</t>
         </is>
       </c>
       <c r="AE10" s="12" t="inlineStr">
         <is>
-          <t>N/A (1 VM/core)</t>
+          <t>Delegated to tenant</t>
         </is>
       </c>
       <c r="AF10" s="12" t="inlineStr">
         <is>
-          <t>N/A (1 VM/core)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AG10" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH10" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Resource-scoped interfaces</t>
         </is>
       </c>
       <c r="AI10" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ10" s="12" t="inlineStr">
         <is>
-          <t>Resource-scoped interfaces</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK10" s="12" t="inlineStr">
@@ -3138,35 +3038,25 @@
       </c>
       <c r="AL10" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AM10" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AN10" s="12" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AO10" s="12" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="AO10" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="AP10" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AQ10" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="AR10" s="12" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -3268,12 +3158,12 @@
       </c>
       <c r="T11" s="12" t="inlineStr">
         <is>
-          <t>Dynamic</t>
+          <t>MPU (dynamic)</t>
         </is>
       </c>
       <c r="U11" s="12" t="inlineStr">
         <is>
-          <t>MPU</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V11" s="12" t="inlineStr">
@@ -3288,7 +3178,7 @@
       </c>
       <c r="X11" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MPU fault handler</t>
         </is>
       </c>
       <c r="Y11" s="12" t="inlineStr">
@@ -3298,7 +3188,7 @@
       </c>
       <c r="Z11" s="12" t="inlineStr">
         <is>
-          <t>MPU fault handler</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AA11" s="12" t="inlineStr">
@@ -3323,70 +3213,60 @@
       </c>
       <c r="AE11" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AF11" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="AG11" s="12" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH11" s="12" t="inlineStr">
+        <is>
+          <t>Resource-scoped interfaces</t>
+        </is>
+      </c>
+      <c r="AI11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AL11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AM11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AN11" s="12" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH11" s="12" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="AI11" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AJ11" s="12" t="inlineStr">
-        <is>
-          <t>Resource-scoped interfaces</t>
-        </is>
-      </c>
-      <c r="AK11" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AL11" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AM11" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AN11" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="AO11" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="AP11" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ11" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR11" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3488,97 +3368,97 @@
       </c>
       <c r="T12" s="12" t="inlineStr">
         <is>
-          <t>Dynamic</t>
+          <t>MPU (dynamic)</t>
         </is>
       </c>
       <c r="U12" s="12" t="inlineStr">
         <is>
-          <t>MPU</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V12" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Virtualization: Dedicated core for interrupt handling and interrupt injection</t>
         </is>
       </c>
       <c r="W12" s="12" t="inlineStr">
         <is>
-          <t>Virtualization</t>
+          <t>Hypercall</t>
         </is>
       </c>
       <c r="X12" s="12" t="inlineStr">
         <is>
-          <t>Dedicated core for interrupt handling and interrupt injection</t>
+          <t>HPV-centralized</t>
         </is>
       </c>
       <c r="Y12" s="12" t="inlineStr">
         <is>
-          <t>Hypercall</t>
+          <t>Driver partition</t>
         </is>
       </c>
       <c r="Z12" s="12" t="inlineStr">
         <is>
-          <t>HPV-centralized</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AA12" s="12" t="inlineStr">
         <is>
-          <t>Driver partition</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="AB12" s="12" t="inlineStr">
         <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="AC12" s="12" t="inlineStr">
+        <is>
+          <t>Budget-based</t>
+        </is>
+      </c>
+      <c r="AD12" s="12" t="inlineStr">
+        <is>
+          <t>Budget-based</t>
+        </is>
+      </c>
+      <c r="AE12" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF12" s="12" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AC12" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD12" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE12" s="12" t="inlineStr">
-        <is>
-          <t>Budget-based</t>
-        </is>
-      </c>
-      <c r="AF12" s="12" t="inlineStr">
-        <is>
-          <t>Budget-based</t>
-        </is>
-      </c>
       <c r="AG12" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH12" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Proprietary hypervisor APIs</t>
         </is>
       </c>
       <c r="AI12" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AJ12" s="12" t="inlineStr">
         <is>
-          <t>Proprietary hypervisor APIs</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AK12" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AL12" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AM12" s="12" t="inlineStr">
@@ -3588,7 +3468,7 @@
       </c>
       <c r="AN12" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO12" s="12" t="inlineStr">
@@ -3597,16 +3477,6 @@
         </is>
       </c>
       <c r="AP12" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ12" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR12" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3708,87 +3578,87 @@
       </c>
       <c r="T13" s="12" t="inlineStr">
         <is>
-          <t>Dynamic</t>
+          <t>MPU (dynamic)</t>
         </is>
       </c>
       <c r="U13" s="12" t="inlineStr">
         <is>
-          <t>MPU</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V13" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Virtualization: Virtual interrupt injection</t>
         </is>
       </c>
       <c r="W13" s="12" t="inlineStr">
         <is>
-          <t>Virtualization</t>
+          <t>Hypercall</t>
         </is>
       </c>
       <c r="X13" s="12" t="inlineStr">
         <is>
-          <t>Virtual interrupt injection</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="Y13" s="12" t="inlineStr">
         <is>
-          <t>Hypercall</t>
+          <t>DDA + Paravirtualization</t>
         </is>
       </c>
       <c r="Z13" s="12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA13" s="12" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="AA13" s="12" t="inlineStr">
-        <is>
-          <t>DDA + Paravirtualization</t>
-        </is>
-      </c>
       <c r="AB13" s="12" t="inlineStr">
         <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="AC13" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to host RTOS</t>
+        </is>
+      </c>
+      <c r="AD13" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to host RTOS</t>
+        </is>
+      </c>
+      <c r="AE13" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF13" s="12" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AC13" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD13" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE13" s="12" t="inlineStr">
-        <is>
-          <t>Delegated to host RTOS</t>
-        </is>
-      </c>
-      <c r="AF13" s="12" t="inlineStr">
-        <is>
-          <t>Delegated to host RTOS</t>
-        </is>
-      </c>
       <c r="AG13" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AH13" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Proprietary hypervisor APIs</t>
         </is>
       </c>
       <c r="AI13" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ13" s="12" t="inlineStr">
         <is>
-          <t>Proprietary hypervisor APIs</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AK13" s="12" t="inlineStr">
@@ -3803,30 +3673,20 @@
       </c>
       <c r="AM13" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AN13" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO13" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AP13" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ13" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR13" s="12" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -3928,87 +3788,87 @@
       </c>
       <c r="T14" s="12" t="inlineStr">
         <is>
-          <t>Dynamic</t>
+          <t>MPU + TrustZone-M (dynamic)</t>
         </is>
       </c>
       <c r="U14" s="12" t="inlineStr">
         <is>
-          <t>MPU + TrustZone-M</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V14" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Hybrid: Virtual interrupt injection + SBI bypass</t>
         </is>
       </c>
       <c r="W14" s="12" t="inlineStr">
         <is>
-          <t>Hybrid</t>
+          <t>Hypercall</t>
         </is>
       </c>
       <c r="X14" s="12" t="inlineStr">
         <is>
-          <t>Virtual interrupt injection + SBI bypass</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="Y14" s="12" t="inlineStr">
         <is>
-          <t>Hypercall</t>
+          <t>DDA + Driver partition</t>
         </is>
       </c>
       <c r="Z14" s="12" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA14" s="12" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="AA14" s="12" t="inlineStr">
-        <is>
-          <t>DDA + Driver partition</t>
-        </is>
-      </c>
       <c r="AB14" s="12" t="inlineStr">
         <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="AC14" s="12" t="inlineStr">
+        <is>
+          <t>Fixed-priority preemptive</t>
+        </is>
+      </c>
+      <c r="AD14" s="12" t="inlineStr">
+        <is>
+          <t>Fixed-priority preemptive</t>
+        </is>
+      </c>
+      <c r="AE14" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF14" s="12" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AC14" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD14" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE14" s="12" t="inlineStr">
-        <is>
-          <t>Fixed-priority preemptive</t>
-        </is>
-      </c>
-      <c r="AF14" s="12" t="inlineStr">
-        <is>
-          <t>Fixed-priority preemptive</t>
-        </is>
-      </c>
       <c r="AG14" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AH14" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Proprietary hypervisor APIs</t>
         </is>
       </c>
       <c r="AI14" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ14" s="12" t="inlineStr">
         <is>
-          <t>Proprietary hypervisor APIs</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK14" s="12" t="inlineStr">
@@ -4018,35 +3878,25 @@
       </c>
       <c r="AL14" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AM14" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AN14" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO14" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AP14" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ14" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR14" s="12" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -4163,92 +4013,92 @@
       </c>
       <c r="W15" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="X15" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="Y15" s="12" t="inlineStr">
         <is>
+          <t>HW I/O virtualization</t>
+        </is>
+      </c>
+      <c r="Z15" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA15" s="12" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="Z15" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AA15" s="12" t="inlineStr">
-        <is>
-          <t>HW I/O virtualization</t>
-        </is>
-      </c>
       <c r="AB15" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Static</t>
         </is>
       </c>
       <c r="AC15" s="12" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>N/A (1 VM/core)</t>
         </is>
       </c>
       <c r="AD15" s="12" t="inlineStr">
         <is>
-          <t>Static</t>
+          <t>N/A (1 VM/core)</t>
         </is>
       </c>
       <c r="AE15" s="12" t="inlineStr">
         <is>
-          <t>N/A (1 VM/core)</t>
+          <t>Delegated to tenant</t>
         </is>
       </c>
       <c r="AF15" s="12" t="inlineStr">
         <is>
-          <t>N/A (1 VM/core)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AG15" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH15" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Resource-scoped interfaces</t>
         </is>
       </c>
       <c r="AI15" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AJ15" s="12" t="inlineStr">
         <is>
-          <t>Resource-scoped interfaces</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK15" s="12" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AL15" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AM15" s="12" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="AL15" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AM15" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="AN15" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AO15" s="12" t="inlineStr">
@@ -4257,16 +4107,6 @@
         </is>
       </c>
       <c r="AP15" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="AQ15" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="AR15" s="12" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -4364,72 +4204,72 @@
       </c>
       <c r="T16" s="12" t="inlineStr">
         <is>
-          <t>Static</t>
+          <t>XMPU/XPPU (static)</t>
         </is>
       </c>
       <c r="U16" s="12" t="inlineStr">
         <is>
-          <t>XMPU/XPPU</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V16" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Direct Access: HW core isolation</t>
         </is>
       </c>
       <c r="W16" s="12" t="inlineStr">
         <is>
-          <t>Direct Access</t>
+          <t>None</t>
         </is>
       </c>
       <c r="X16" s="12" t="inlineStr">
         <is>
-          <t>HW core isolation</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="Y16" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>DDA (pass-through)</t>
         </is>
       </c>
       <c r="Z16" s="12" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA16" s="12" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="AA16" s="12" t="inlineStr">
-        <is>
-          <t>DDA (pass-through)</t>
-        </is>
-      </c>
       <c r="AB16" s="12" t="inlineStr">
         <is>
+          <t>Dynamic</t>
+        </is>
+      </c>
+      <c r="AC16" s="12" t="inlineStr">
+        <is>
+          <t>N/A (1 VM/core)</t>
+        </is>
+      </c>
+      <c r="AD16" s="12" t="inlineStr">
+        <is>
+          <t>N/A (1 VM/core)</t>
+        </is>
+      </c>
+      <c r="AE16" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF16" s="12" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AC16" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD16" s="12" t="inlineStr">
-        <is>
-          <t>Dynamic</t>
-        </is>
-      </c>
-      <c r="AE16" s="12" t="inlineStr">
-        <is>
-          <t>N/A (1 VM/core)</t>
-        </is>
-      </c>
-      <c r="AF16" s="12" t="inlineStr">
-        <is>
-          <t>N/A (1 VM/core)</t>
-        </is>
-      </c>
       <c r="AG16" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH16" s="12" t="inlineStr">
@@ -4439,17 +4279,17 @@
       </c>
       <c r="AI16" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AJ16" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK16" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AL16" s="12" t="inlineStr">
@@ -4464,7 +4304,7 @@
       </c>
       <c r="AN16" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO16" s="12" t="inlineStr">
@@ -4473,16 +4313,6 @@
         </is>
       </c>
       <c r="AP16" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ16" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR16" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4584,72 +4414,72 @@
       </c>
       <c r="T17" s="12" t="inlineStr">
         <is>
+          <t>XMPU/XPPU (static)</t>
+        </is>
+      </c>
+      <c r="U17" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V17" s="12" t="inlineStr">
+        <is>
+          <t>Direct Access: HW core isolation</t>
+        </is>
+      </c>
+      <c r="W17" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="X17" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="Y17" s="12" t="inlineStr">
+        <is>
+          <t>DDA (pass-through)</t>
+        </is>
+      </c>
+      <c r="Z17" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA17" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="AB17" s="12" t="inlineStr">
+        <is>
           <t>Static</t>
         </is>
       </c>
-      <c r="U17" s="12" t="inlineStr">
-        <is>
-          <t>XMPU/XPPU</t>
-        </is>
-      </c>
-      <c r="V17" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W17" s="12" t="inlineStr">
-        <is>
-          <t>Direct Access</t>
-        </is>
-      </c>
-      <c r="X17" s="12" t="inlineStr">
-        <is>
-          <t>HW core isolation</t>
-        </is>
-      </c>
-      <c r="Y17" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z17" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AA17" s="12" t="inlineStr">
-        <is>
-          <t>DDA (pass-through)</t>
-        </is>
-      </c>
-      <c r="AB17" s="12" t="inlineStr">
+      <c r="AC17" s="12" t="inlineStr">
+        <is>
+          <t>N/A (1 VM/core)</t>
+        </is>
+      </c>
+      <c r="AD17" s="12" t="inlineStr">
+        <is>
+          <t>N/A (1 VM/core)</t>
+        </is>
+      </c>
+      <c r="AE17" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF17" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AC17" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD17" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE17" s="12" t="inlineStr">
-        <is>
-          <t>N/A (1 VM/core)</t>
-        </is>
-      </c>
-      <c r="AF17" s="12" t="inlineStr">
-        <is>
-          <t>N/A (1 VM/core)</t>
-        </is>
-      </c>
       <c r="AG17" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH17" s="12" t="inlineStr">
@@ -4659,12 +4489,12 @@
       </c>
       <c r="AI17" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ17" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK17" s="12" t="inlineStr">
@@ -4684,7 +4514,7 @@
       </c>
       <c r="AN17" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO17" s="12" t="inlineStr">
@@ -4693,16 +4523,6 @@
         </is>
       </c>
       <c r="AP17" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ17" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR17" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4804,72 +4624,72 @@
       </c>
       <c r="T18" s="12" t="inlineStr">
         <is>
-          <t>Dynamic</t>
+          <t>MPU + HW ext. (dynamic)</t>
         </is>
       </c>
       <c r="U18" s="12" t="inlineStr">
         <is>
-          <t>MPU + HW ext.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V18" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Direct Access: HW guest attribution</t>
         </is>
       </c>
       <c r="W18" s="12" t="inlineStr">
         <is>
-          <t>Direct Access</t>
+          <t>None</t>
         </is>
       </c>
       <c r="X18" s="12" t="inlineStr">
         <is>
-          <t>HW guest attribution</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="Y18" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>DDA (pass-through)</t>
         </is>
       </c>
       <c r="Z18" s="12" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA18" s="12" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="AA18" s="12" t="inlineStr">
-        <is>
-          <t>DDA (pass-through)</t>
-        </is>
-      </c>
       <c r="AB18" s="12" t="inlineStr">
         <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="AC18" s="12" t="inlineStr">
+        <is>
+          <t>Static time partitioning / Fixed-priority preemptive</t>
+        </is>
+      </c>
+      <c r="AD18" s="12" t="inlineStr">
+        <is>
+          <t>Static time partitioning / Fixed-priority preemptive</t>
+        </is>
+      </c>
+      <c r="AE18" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF18" s="12" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AC18" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD18" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE18" s="12" t="inlineStr">
-        <is>
-          <t>Static time partitioning / Fixed-priority preemptive</t>
-        </is>
-      </c>
-      <c r="AF18" s="12" t="inlineStr">
-        <is>
-          <t>Static time partitioning / Fixed-priority preemptive</t>
-        </is>
-      </c>
       <c r="AG18" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH18" s="12" t="inlineStr">
@@ -4879,12 +4699,12 @@
       </c>
       <c r="AI18" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ18" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AK18" s="12" t="inlineStr">
@@ -4913,16 +4733,6 @@
         </is>
       </c>
       <c r="AP18" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="AQ18" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR18" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5024,87 +4834,87 @@
       </c>
       <c r="T19" s="12" t="inlineStr">
         <is>
+          <t>MPU (static)</t>
+        </is>
+      </c>
+      <c r="U19" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V19" s="12" t="inlineStr">
+        <is>
+          <t>Virtualization: Virtual interrupt injection</t>
+        </is>
+      </c>
+      <c r="W19" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="X19" s="12" t="inlineStr">
+        <is>
+          <t>HPV fault thread + watchdogs</t>
+        </is>
+      </c>
+      <c r="Y19" s="12" t="inlineStr">
+        <is>
+          <t>DDA + Driver VM/process</t>
+        </is>
+      </c>
+      <c r="Z19" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA19" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="AB19" s="12" t="inlineStr">
+        <is>
           <t>Static</t>
         </is>
       </c>
-      <c r="U19" s="12" t="inlineStr">
-        <is>
-          <t>MPU</t>
-        </is>
-      </c>
-      <c r="V19" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W19" s="12" t="inlineStr">
-        <is>
-          <t>Virtualization</t>
-        </is>
-      </c>
-      <c r="X19" s="12" t="inlineStr">
-        <is>
-          <t>Virtual interrupt injection</t>
-        </is>
-      </c>
-      <c r="Y19" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z19" s="12" t="inlineStr">
-        <is>
-          <t>HPV fault thread + watchdogs</t>
-        </is>
-      </c>
-      <c r="AA19" s="12" t="inlineStr">
-        <is>
-          <t>DDA + Driver VM/process</t>
-        </is>
-      </c>
-      <c r="AB19" s="12" t="inlineStr">
+      <c r="AC19" s="12" t="inlineStr">
+        <is>
+          <t>Fixed-priority preemptive</t>
+        </is>
+      </c>
+      <c r="AD19" s="12" t="inlineStr">
+        <is>
+          <t>Fixed-priority preemptive</t>
+        </is>
+      </c>
+      <c r="AE19" s="12" t="inlineStr">
+        <is>
+          <t>Delegated to tenant</t>
+        </is>
+      </c>
+      <c r="AF19" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="AC19" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD19" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE19" s="12" t="inlineStr">
-        <is>
-          <t>Fixed-priority preemptive</t>
-        </is>
-      </c>
-      <c r="AF19" s="12" t="inlineStr">
-        <is>
-          <t>Fixed-priority preemptive</t>
-        </is>
-      </c>
       <c r="AG19" s="12" t="inlineStr">
         <is>
-          <t>Delegated to tenant</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AH19" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Proprietary hypervisor APIs</t>
         </is>
       </c>
       <c r="AI19" s="12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ19" s="12" t="inlineStr">
         <is>
-          <t>Proprietary hypervisor APIs</t>
+          <t>●</t>
         </is>
       </c>
       <c r="AK19" s="12" t="inlineStr">
@@ -5124,25 +4934,15 @@
       </c>
       <c r="AN19" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AO19" s="12" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="AO19" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="AP19" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ19" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="AR19" s="12" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -5244,87 +5044,87 @@
       </c>
       <c r="T20" s="12" t="inlineStr">
         <is>
-          <t>Dynamic</t>
+          <t>MPU (dynamic)</t>
         </is>
       </c>
       <c r="U20" s="12" t="inlineStr">
         <is>
-          <t>MPU</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V20" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Partitioning: Virtualization layer-mediated forwarding</t>
         </is>
       </c>
       <c r="W20" s="12" t="inlineStr">
         <is>
-          <t>Partitioning</t>
+          <t>Hypercall</t>
         </is>
       </c>
       <c r="X20" s="12" t="inlineStr">
         <is>
-          <t>Virtualization layer-mediated forwarding</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="Y20" s="12" t="inlineStr">
         <is>
-          <t>Hypercall</t>
+          <t>Virtualization layer-managed</t>
         </is>
       </c>
       <c r="Z20" s="12" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA20" s="12" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="AA20" s="12" t="inlineStr">
-        <is>
-          <t>Virtualization layer-managed</t>
-        </is>
-      </c>
       <c r="AB20" s="12" t="inlineStr">
         <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="AC20" s="12" t="inlineStr">
+        <is>
+          <t>Static time partitioning</t>
+        </is>
+      </c>
+      <c r="AD20" s="12" t="inlineStr">
+        <is>
+          <t>Static time partitioning</t>
+        </is>
+      </c>
+      <c r="AE20" s="12" t="inlineStr">
+        <is>
+          <t>Managed by virtualization layer</t>
+        </is>
+      </c>
+      <c r="AF20" s="12" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="AC20" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AD20" s="12" t="inlineStr">
-        <is>
-          <t>Static</t>
-        </is>
-      </c>
-      <c r="AE20" s="12" t="inlineStr">
-        <is>
-          <t>Static time partitioning</t>
-        </is>
-      </c>
-      <c r="AF20" s="12" t="inlineStr">
-        <is>
-          <t>Static time partitioning</t>
-        </is>
-      </c>
       <c r="AG20" s="12" t="inlineStr">
         <is>
-          <t>Managed by virtualization layer</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AH20" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Standard middleware APIs</t>
         </is>
       </c>
       <c r="AI20" s="12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AJ20" s="12" t="inlineStr">
         <is>
-          <t>Standard middleware APIs</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AK20" s="12" t="inlineStr">
@@ -5344,7 +5144,7 @@
       </c>
       <c r="AN20" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AO20" s="12" t="inlineStr">
@@ -5353,16 +5153,6 @@
         </is>
       </c>
       <c r="AP20" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ20" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR20" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5464,125 +5254,115 @@
       </c>
       <c r="T21" s="12" t="inlineStr">
         <is>
+          <t>MPU (static)</t>
+        </is>
+      </c>
+      <c r="U21" s="12" t="inlineStr">
+        <is>
+          <t>Wasm</t>
+        </is>
+      </c>
+      <c r="V21" s="12" t="inlineStr">
+        <is>
+          <t>Partitioning: Virtualization layer-mediated forwarding</t>
+        </is>
+      </c>
+      <c r="W21" s="12" t="inlineStr">
+        <is>
+          <t>Runtime Interposition/Hypercall</t>
+        </is>
+      </c>
+      <c r="X21" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="Y21" s="12" t="inlineStr">
+        <is>
+          <t>Paravirtualization + Trap-and-emulate (no full virtualization)</t>
+        </is>
+      </c>
+      <c r="Z21" s="12" t="inlineStr">
+        <is>
+          <t>Not evaluated</t>
+        </is>
+      </c>
+      <c r="AA21" s="12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="AB21" s="12" t="inlineStr">
+        <is>
           <t>Static</t>
         </is>
       </c>
-      <c r="U21" s="12" t="inlineStr">
-        <is>
-          <t>MPU</t>
-        </is>
-      </c>
-      <c r="V21" s="12" t="inlineStr">
-        <is>
-          <t>Wasm</t>
-        </is>
-      </c>
-      <c r="W21" s="12" t="inlineStr">
-        <is>
-          <t>Partitioning</t>
-        </is>
-      </c>
-      <c r="X21" s="12" t="inlineStr">
-        <is>
-          <t>Virtualization layer-mediated forwarding</t>
-        </is>
-      </c>
-      <c r="Y21" s="12" t="inlineStr">
-        <is>
-          <t>Runtime Interposition/Hypercall</t>
-        </is>
-      </c>
-      <c r="Z21" s="12" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AA21" s="12" t="inlineStr">
-        <is>
-          <t>Paravirtualization + Trap-and-emulate (no full virtualization)</t>
-        </is>
-      </c>
-      <c r="AB21" s="12" t="inlineStr">
-        <is>
-          <t>Not evaluated</t>
-        </is>
-      </c>
       <c r="AC21" s="12" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Delegated to host RTOS</t>
         </is>
       </c>
       <c r="AD21" s="12" t="inlineStr">
         <is>
-          <t>Static</t>
+          <t>Delegated to host RTOS</t>
         </is>
       </c>
       <c r="AE21" s="12" t="inlineStr">
         <is>
-          <t>Delegated to host RTOS</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="AF21" s="12" t="inlineStr">
         <is>
-          <t>Delegated to host RTOS</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AG21" s="12" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH21" s="12" t="inlineStr">
+        <is>
+          <t>Resource-scoped interfaces</t>
+        </is>
+      </c>
+      <c r="AI21" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ21" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK21" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AL21" s="12" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="AM21" s="12" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="AN21" s="12" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="AH21" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AI21" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AJ21" s="12" t="inlineStr">
-        <is>
-          <t>Resource-scoped interfaces</t>
-        </is>
-      </c>
-      <c r="AK21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AL21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AM21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AN21" s="12" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
       <c r="AO21" s="12" t="inlineStr">
         <is>
-          <t>●</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AP21" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AQ21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AR21" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5591,14 +5371,14 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="G1:L1"/>
-    <mergeCell ref="T1:V1"/>
     <mergeCell ref="M1:S1"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="AA1:AB1"/>
-    <mergeCell ref="AK1:AR1"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="AE1:AH1"/>
+    <mergeCell ref="Y1:Z1"/>
+    <mergeCell ref="AI1:AP1"/>
+    <mergeCell ref="AA1:AD1"/>
+    <mergeCell ref="V1:X1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>